<commit_message>
tests hechos para multicliente
</commit_message>
<xml_diff>
--- a/src/main/resources/client-packinglist/ami-belts-packing-list-template.xlsx
+++ b/src/main/resources/client-packinglist/ami-belts-packing-list-template.xlsx
@@ -15,6 +15,7 @@
   <sheets>
     <sheet name="Tableau1" sheetId="2" state="hidden" r:id="rId1"/>
     <sheet name="STANDARD PKL E25" sheetId="1" r:id="rId2"/>
+    <sheet name="Feuil1" r:id="rId12" sheetId="3" state="hidden"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'STANDARD PKL E25'!$A$1:$U$28</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="78">
   <si>
     <t>ORDER FORM NUMBER</t>
   </si>
@@ -317,6 +318,18 @@
   </si>
   <si>
     <t>85-95-105</t>
+  </si>
+  <si>
+    <t>DESTINATION</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Hong Kong</t>
+  </si>
+  <si>
+    <t>Japan</t>
   </si>
 </sst>
 </file>
@@ -1918,6 +1931,11 @@
     <mergeCell ref="A1:U1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="B10" allowBlank="true" errorStyle="stop" showErrorMessage="true">
+      <formula1>Feuil1!$A$2:$A$5</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.74803149606299213" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="64" orientation="landscape" r:id="rId1"/>
@@ -1925,6 +1943,41 @@
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 

</xml_diff>